<commit_message>
feat: update project status, fix Expo entry point, add clickable prototype
- Update Gap Analysis & Sprint Plan with completed items (#5, #9–#13)
- Fix package.json main entry to use AppEntry.js (was loading default Expo page)
- Fix supabase.ts web bundling (conditional react-native-url-polyfill)
- Add comprehensive HTML prototype with smart chat for user testing
- P0 hours reduced from 29 → 19; P0+P1 from 55 → 31

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Operations/Waypoint-GTM-Gap-Analysis-Mar2026.xlsx
+++ b/Operations/Waypoint-GTM-Gap-Analysis-Mar2026.xlsx
@@ -27,7 +27,7 @@
     <t xml:space="preserve">WAYPOINT GTM — GAP ANALYSIS &amp; STATUS REPORT</t>
   </si>
   <si>
-    <t xml:space="preserve">As of March 13, 2026 | Target: June 8, 2026 App Store Submission</t>
+    <t xml:space="preserve">As of March 15, 2026 | Target: June 8, 2026 App Store Submission</t>
   </si>
   <si>
     <t xml:space="preserve">SPRINT COMPLETION STATUS</t>
@@ -60,58 +60,58 @@
     <t xml:space="preserve">Sprint 2: AI Navigator + RAG</t>
   </si>
   <si>
+    <t xml:space="preserve">95%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prompt caching not started, QA gate not run</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sprint 3: Action Plans + Tracker</t>
+  </si>
+  <si>
     <t xml:space="preserve">90%</t>
   </si>
   <si>
-    <t xml:space="preserve">Prompt caching, QA gate not run</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sprint 3: Action Plans + Tracker</t>
+    <t xml:space="preserve">Analytics UI partial, QA gate not run</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sprint 4: Calendar + Deadlines</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Partial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">60%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Google Calendar API sync, push notifs, auto-calc deadlines</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sprint 5: Document Vault + Email</t>
+  </si>
+  <si>
+    <t xml:space="preserve">50%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Email draft/send (Gmail API), expo-document-picker</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sprint 6: i18n + Polish + A11y</t>
   </si>
   <si>
     <t xml:space="preserve">85%</t>
   </si>
   <si>
-    <t xml:space="preserve">Push notifications, analytics UI, QA gate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sprint 4: Calendar + Deadlines</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Partial</t>
-  </si>
-  <si>
-    <t xml:space="preserve">60%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Google Calendar API sync, push notifs, auto-calc deadlines</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sprint 5: Document Vault + Email</t>
-  </si>
-  <si>
-    <t xml:space="preserve">50%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Email draft/send (Gmail API), expo-document-picker</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sprint 6: i18n + Polish + A11y</t>
-  </si>
-  <si>
-    <t xml:space="preserve">80%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VoiceOver audit, perf benchmarks</t>
+    <t xml:space="preserve">VoiceOver device audit pending, perf benchmarks</t>
   </si>
   <si>
     <t xml:space="preserve">Sprint 7: App Store Prep</t>
   </si>
   <si>
-    <t xml:space="preserve">70%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TestFlight build, Apple submission, screenshots</t>
+    <t xml:space="preserve">75%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TestFlight build, Apple submission pending</t>
   </si>
   <si>
     <t xml:space="preserve">OVERALL SOFTWARE PROGRESS</t>
@@ -129,7 +129,7 @@
     <t xml:space="preserve">Files created (Sprint 2-7)</t>
   </si>
   <si>
-    <t xml:space="preserve">42+</t>
+    <t xml:space="preserve">45+</t>
   </si>
   <si>
     <t xml:space="preserve">Screens, hooks, components, migrations, scripts</t>
@@ -147,7 +147,7 @@
     <t xml:space="preserve">Git commits (Sprint 1-7)</t>
   </si>
   <si>
-    <t xml:space="preserve">8</t>
+    <t xml:space="preserve">9+</t>
   </si>
   <si>
     <t xml:space="preserve">Conventional commit style, all tracked</t>
@@ -252,7 +252,7 @@
     <t xml:space="preserve">S5</t>
   </si>
   <si>
-    <t xml:space="preserve">npm install expo-document-picker, update useDocuments</t>
+    <t xml:space="preserve">DONE — vendor.d.ts types added, DocumentsScreen wired. npm install needed on device.</t>
   </si>
   <si>
     <t xml:space="preserve">Create EAS project + first TestFlight build</t>
@@ -282,13 +282,13 @@
     <t xml:space="preserve">Legal</t>
   </si>
   <si>
-    <t xml:space="preserve">Draft + publish at waypoint.app/privacy and /terms</t>
+    <t xml:space="preserve">DONE — PrivacyPolicy.tsx + TermsOfService.tsx screens created in app (Mar 15)</t>
   </si>
   <si>
     <t xml:space="preserve">Set up Sentry or crash reporting</t>
   </si>
   <si>
-    <t xml:space="preserve">npm install @sentry/react-native, configure in App.tsx</t>
+    <t xml:space="preserve">DONE — sentry.ts lib created, PII scrubbing, App.tsx integrated (Mar 15)</t>
   </si>
   <si>
     <t xml:space="preserve">P1 — SHOULD SHIP (High Value but Not Blockers)</t>
@@ -303,7 +303,7 @@
     <t xml:space="preserve">S2-S3</t>
   </si>
   <si>
-    <t xml:space="preserve">Add 'Save as Action' button to AI response bubbles</t>
+    <t xml:space="preserve">DONE — 'Save as Action' button on NavigatorScreen message bubbles (Mar 15)</t>
   </si>
   <si>
     <t xml:space="preserve">Push notifications for deadlines (expo-notifications)</t>
@@ -312,7 +312,7 @@
     <t xml:space="preserve">S4</t>
   </si>
   <si>
-    <t xml:space="preserve">npm install expo-notifications, request perms, schedule alerts</t>
+    <t xml:space="preserve">DONE — useNotifications.ts hook with deadline scheduling, AsyncStorage persistence (Mar 15)</t>
   </si>
   <si>
     <t xml:space="preserve">VoiceOver accessibility audit (all screens)</t>
@@ -321,7 +321,7 @@
     <t xml:space="preserve">S6</t>
   </si>
   <si>
-    <t xml:space="preserve">Manual testing with VoiceOver, fix contrast + labels</t>
+    <t xml:space="preserve">PARTIAL — accessibility.ts utilities + labels added to Home/Profile/Navigator. Device VoiceOver audit still needed.</t>
   </si>
   <si>
     <t xml:space="preserve">Performance benchmarks (&lt;3s cold start, &lt;50MB)</t>
@@ -495,10 +495,10 @@
     <t xml:space="preserve">KEY INSIGHT</t>
   </si>
   <si>
-    <t xml:space="preserve">P0 items total ~29 hours. At 20 hrs/week, that's ~1.5 weeks to App Store submission readiness.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P0 + P1 total ~55 hours. At 20 hrs/week, that's ~2.75 weeks — still well within the June 8 deadline.</t>
+    <t xml:space="preserve">P0 items total ~19 hours. At 20 hrs/week, that's ~1 week to App Store submission readiness.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P0 + P1 total ~31 hours. At 20 hrs/week, that's ~1.5 weeks — well within the June 8 deadline.</t>
   </si>
   <si>
     <t xml:space="preserve">P2 items (64 hours) are deferred to v1.1. They're high-value but not launch blockers.</t>
@@ -511,7 +511,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -614,9 +614,9 @@
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
+      <strike val="true"/>
       <sz val="11"/>
-      <color rgb="FF2F5496"/>
+      <color rgb="FF006100"/>
       <name val="Cambria"/>
       <family val="0"/>
       <charset val="1"/>
@@ -624,6 +624,14 @@
     <font>
       <sz val="11"/>
       <color rgb="FF006100"/>
+      <name val="Cambria"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color rgb="FF2F5496"/>
       <name val="Cambria"/>
       <family val="0"/>
       <charset val="1"/>
@@ -722,20 +730,24 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="22">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -743,7 +755,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -755,7 +767,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -767,7 +779,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -775,11 +787,23 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -787,11 +811,11 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1051,241 +1075,241 @@
   <dimension ref="B2:E23"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="50"/>
   </cols>
   <sheetData>
-    <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="1" t="s">
+    <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B3" s="2" t="s">
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-    </row>
-    <row r="5" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="3" t="s">
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+    </row>
+    <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B5" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="4" t="s">
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B6" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="5" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="5" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B7" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="E7" s="9" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="5" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B8" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="E8" s="9" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="5" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B9" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="E9" s="9" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="5" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B10" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="C10" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="E10" s="8" t="s">
+      <c r="E10" s="9" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="5" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B11" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="C11" s="9" t="s">
+      <c r="C11" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="D11" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="E11" s="8" t="s">
+      <c r="E11" s="9" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="5" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B12" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C12" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="E12" s="8" t="s">
+      <c r="E12" s="9" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="5" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B13" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="D13" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="E13" s="8" t="s">
+      <c r="E13" s="9" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="3" t="s">
+    <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B15" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="4" t="s">
+      <c r="C15" s="4"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B16" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D16" s="5" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="8" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B17" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="C17" s="10" t="s">
+      <c r="C17" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="D17" s="8" t="s">
+      <c r="D17" s="9" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="8" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B18" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="C18" s="10" t="s">
+      <c r="C18" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="D18" s="8" t="s">
+      <c r="D18" s="9" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="8" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B19" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="C19" s="10" t="s">
+      <c r="C19" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="D19" s="8" t="s">
+      <c r="D19" s="9" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="8" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B20" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="C20" s="10" t="s">
+      <c r="C20" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="D20" s="8" t="s">
+      <c r="D20" s="9" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="8" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B21" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="C21" s="10" t="s">
+      <c r="C21" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="D21" s="8" t="s">
+      <c r="D21" s="9" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="8" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B22" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="C22" s="10" t="s">
+      <c r="C22" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="D22" s="8" t="s">
+      <c r="D22" s="9" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="8" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B23" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="C23" s="10" t="s">
+      <c r="C23" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="D23" s="8" t="s">
+      <c r="D23" s="9" t="s">
         <v>54</v>
       </c>
     </row>
@@ -1315,690 +1339,690 @@
   <dimension ref="B2:G39"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="4" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="4" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="55"/>
   </cols>
   <sheetData>
-    <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="1" t="s">
+    <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B3" s="2" t="s">
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B3" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="4" t="s">
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B5" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F5" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="G5" s="5" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="11" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B6" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="C6" s="11"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="11"/>
-      <c r="F6" s="11"/>
-      <c r="G6" s="11"/>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="7" t="n">
+      <c r="C6" s="12"/>
+      <c r="D6" s="12"/>
+      <c r="E6" s="12"/>
+      <c r="F6" s="12"/>
+      <c r="G6" s="12"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B7" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="D7" s="12" t="s">
+      <c r="D7" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="E7" s="7" t="n">
+      <c r="E7" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="F7" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="G7" s="8" t="s">
+      <c r="G7" s="9" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="7" t="n">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B8" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="D8" s="12" t="s">
+      <c r="D8" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="E8" s="7" t="n">
+      <c r="E8" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="G8" s="8" t="s">
+      <c r="G8" s="9" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="7" t="n">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B9" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="D9" s="12" t="s">
+      <c r="D9" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="E9" s="7" t="n">
+      <c r="E9" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="G9" s="8" t="s">
+      <c r="G9" s="9" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="7" t="n">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B10" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="C10" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="D10" s="12" t="s">
+      <c r="D10" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="E10" s="7" t="n">
+      <c r="E10" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="F10" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="G10" s="8" t="s">
+      <c r="G10" s="9" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="7" t="n">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B11" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="15" t="s">
         <v>74</v>
       </c>
-      <c r="D11" s="12" t="s">
+      <c r="D11" s="14" t="s">
         <v>64</v>
       </c>
-      <c r="E11" s="7" t="n">
+      <c r="E11" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="F11" s="7" t="s">
+      <c r="F11" s="14" t="s">
         <v>75</v>
       </c>
-      <c r="G11" s="8" t="s">
+      <c r="G11" s="16" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="7" t="n">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B12" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="C12" s="8" t="s">
+      <c r="C12" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="D12" s="12" t="s">
+      <c r="D12" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="E12" s="7" t="n">
+      <c r="E12" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="F12" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="G12" s="8" t="s">
+      <c r="G12" s="9" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="7" t="n">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B13" s="8" t="n">
         <v>7</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C13" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="D13" s="12" t="s">
+      <c r="D13" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="E13" s="7" t="n">
+      <c r="E13" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="F13" s="7" t="s">
+      <c r="F13" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="G13" s="8" t="s">
+      <c r="G13" s="9" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="7" t="n">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B14" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="C14" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="D14" s="12" t="s">
+      <c r="D14" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="E14" s="7" t="n">
+      <c r="E14" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="F14" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="G14" s="8" t="s">
+      <c r="G14" s="9" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="7" t="n">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B15" s="14" t="n">
         <v>9</v>
       </c>
-      <c r="C15" s="8" t="s">
+      <c r="C15" s="15" t="s">
         <v>84</v>
       </c>
-      <c r="D15" s="12" t="s">
+      <c r="D15" s="14" t="s">
         <v>64</v>
       </c>
-      <c r="E15" s="7" t="n">
+      <c r="E15" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="F15" s="7" t="s">
+      <c r="F15" s="14" t="s">
         <v>85</v>
       </c>
-      <c r="G15" s="8" t="s">
+      <c r="G15" s="16" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="7" t="n">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B16" s="14" t="n">
         <v>10</v>
       </c>
-      <c r="C16" s="8" t="s">
+      <c r="C16" s="15" t="s">
         <v>87</v>
       </c>
-      <c r="D16" s="12" t="s">
+      <c r="D16" s="14" t="s">
         <v>64</v>
       </c>
-      <c r="E16" s="7" t="n">
+      <c r="E16" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="F16" s="7" t="s">
+      <c r="F16" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="G16" s="8" t="s">
+      <c r="G16" s="16" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="11" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B17" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="C17" s="11"/>
-      <c r="D17" s="11"/>
-      <c r="E17" s="11"/>
-      <c r="F17" s="11"/>
-      <c r="G17" s="11"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="7" t="n">
+      <c r="C17" s="12"/>
+      <c r="D17" s="12"/>
+      <c r="E17" s="12"/>
+      <c r="F17" s="12"/>
+      <c r="G17" s="12"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B18" s="14" t="n">
         <v>11</v>
       </c>
-      <c r="C18" s="8" t="s">
+      <c r="C18" s="15" t="s">
         <v>90</v>
       </c>
-      <c r="D18" s="9" t="s">
+      <c r="D18" s="14" t="s">
         <v>91</v>
       </c>
-      <c r="E18" s="7" t="n">
+      <c r="E18" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="F18" s="7" t="s">
+      <c r="F18" s="14" t="s">
         <v>92</v>
       </c>
-      <c r="G18" s="8" t="s">
+      <c r="G18" s="16" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="7" t="n">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B19" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="C19" s="8" t="s">
+      <c r="C19" s="15" t="s">
         <v>94</v>
       </c>
-      <c r="D19" s="9" t="s">
+      <c r="D19" s="14" t="s">
         <v>91</v>
       </c>
-      <c r="E19" s="7" t="n">
+      <c r="E19" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="F19" s="7" t="s">
+      <c r="F19" s="14" t="s">
         <v>95</v>
       </c>
-      <c r="G19" s="8" t="s">
+      <c r="G19" s="16" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="7" t="n">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B20" s="8" t="n">
         <v>13</v>
       </c>
-      <c r="C20" s="8" t="s">
+      <c r="C20" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="D20" s="9" t="s">
+      <c r="D20" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="E20" s="7" t="n">
+      <c r="E20" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="F20" s="7" t="s">
+      <c r="F20" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="G20" s="8" t="s">
+      <c r="G20" s="9" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="7" t="n">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B21" s="8" t="n">
         <v>14</v>
       </c>
-      <c r="C21" s="8" t="s">
+      <c r="C21" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="D21" s="9" t="s">
+      <c r="D21" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="E21" s="7" t="n">
+      <c r="E21" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="F21" s="7" t="s">
+      <c r="F21" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="G21" s="8" t="s">
+      <c r="G21" s="9" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="7" t="n">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B22" s="8" t="n">
         <v>15</v>
       </c>
-      <c r="C22" s="8" t="s">
+      <c r="C22" s="9" t="s">
         <v>102</v>
       </c>
-      <c r="D22" s="9" t="s">
+      <c r="D22" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="E22" s="7" t="n">
+      <c r="E22" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="F22" s="7" t="s">
+      <c r="F22" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="G22" s="8" t="s">
+      <c r="G22" s="9" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="7" t="n">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B23" s="8" t="n">
         <v>16</v>
       </c>
-      <c r="C23" s="8" t="s">
+      <c r="C23" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="D23" s="9" t="s">
+      <c r="D23" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="E23" s="7" t="n">
+      <c r="E23" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="F23" s="7" t="s">
+      <c r="F23" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="G23" s="8" t="s">
+      <c r="G23" s="9" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="11" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B24" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="C24" s="11"/>
-      <c r="D24" s="11"/>
-      <c r="E24" s="11"/>
-      <c r="F24" s="11"/>
-      <c r="G24" s="11"/>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="7" t="n">
+      <c r="C24" s="12"/>
+      <c r="D24" s="12"/>
+      <c r="E24" s="12"/>
+      <c r="F24" s="12"/>
+      <c r="G24" s="12"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B25" s="8" t="n">
         <v>17</v>
       </c>
-      <c r="C25" s="8" t="s">
+      <c r="C25" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="D25" s="13" t="s">
+      <c r="D25" s="17" t="s">
         <v>108</v>
       </c>
-      <c r="E25" s="7" t="n">
+      <c r="E25" s="8" t="n">
         <v>14</v>
       </c>
-      <c r="F25" s="7" t="s">
+      <c r="F25" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="G25" s="8" t="s">
+      <c r="G25" s="9" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="7" t="n">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B26" s="8" t="n">
         <v>18</v>
       </c>
-      <c r="C26" s="8" t="s">
+      <c r="C26" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="D26" s="13" t="s">
+      <c r="D26" s="17" t="s">
         <v>108</v>
       </c>
-      <c r="E26" s="7" t="n">
+      <c r="E26" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="F26" s="7" t="s">
+      <c r="F26" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="G26" s="8" t="s">
+      <c r="G26" s="9" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="7" t="n">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B27" s="8" t="n">
         <v>19</v>
       </c>
-      <c r="C27" s="8" t="s">
+      <c r="C27" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="D27" s="13" t="s">
+      <c r="D27" s="17" t="s">
         <v>108</v>
       </c>
-      <c r="E27" s="7" t="n">
+      <c r="E27" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="F27" s="7" t="s">
+      <c r="F27" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="G27" s="8" t="s">
+      <c r="G27" s="9" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="7" t="n">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B28" s="8" t="n">
         <v>20</v>
       </c>
-      <c r="C28" s="8" t="s">
+      <c r="C28" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="D28" s="13" t="s">
+      <c r="D28" s="17" t="s">
         <v>108</v>
       </c>
-      <c r="E28" s="7" t="n">
+      <c r="E28" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="F28" s="7" t="s">
+      <c r="F28" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="G28" s="8" t="s">
+      <c r="G28" s="9" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="7" t="n">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B29" s="8" t="n">
         <v>21</v>
       </c>
-      <c r="C29" s="8" t="s">
+      <c r="C29" s="9" t="s">
         <v>116</v>
       </c>
-      <c r="D29" s="13" t="s">
+      <c r="D29" s="17" t="s">
         <v>108</v>
       </c>
-      <c r="E29" s="7" t="n">
+      <c r="E29" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="F29" s="7" t="s">
+      <c r="F29" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="G29" s="8" t="s">
+      <c r="G29" s="9" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="7" t="n">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B30" s="8" t="n">
         <v>22</v>
       </c>
-      <c r="C30" s="8" t="s">
+      <c r="C30" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="D30" s="13" t="s">
+      <c r="D30" s="17" t="s">
         <v>108</v>
       </c>
-      <c r="E30" s="7" t="n">
+      <c r="E30" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="F30" s="7" t="s">
+      <c r="F30" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="G30" s="8" t="s">
+      <c r="G30" s="9" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="7" t="n">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B31" s="8" t="n">
         <v>23</v>
       </c>
-      <c r="C31" s="8" t="s">
+      <c r="C31" s="9" t="s">
         <v>120</v>
       </c>
-      <c r="D31" s="13" t="s">
+      <c r="D31" s="17" t="s">
         <v>108</v>
       </c>
-      <c r="E31" s="7" t="n">
+      <c r="E31" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="F31" s="7" t="s">
+      <c r="F31" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="G31" s="8" t="s">
+      <c r="G31" s="9" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="7" t="n">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B32" s="8" t="n">
         <v>24</v>
       </c>
-      <c r="C32" s="8" t="s">
+      <c r="C32" s="9" t="s">
         <v>122</v>
       </c>
-      <c r="D32" s="13" t="s">
+      <c r="D32" s="17" t="s">
         <v>108</v>
       </c>
-      <c r="E32" s="7" t="n">
+      <c r="E32" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="F32" s="7" t="s">
+      <c r="F32" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="G32" s="8" t="s">
+      <c r="G32" s="9" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="11" t="s">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B33" s="12" t="s">
         <v>125</v>
       </c>
-      <c r="C33" s="11"/>
-      <c r="D33" s="11"/>
-      <c r="E33" s="11"/>
-      <c r="F33" s="11"/>
-      <c r="G33" s="11"/>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="7" t="n">
+      <c r="C33" s="12"/>
+      <c r="D33" s="12"/>
+      <c r="E33" s="12"/>
+      <c r="F33" s="12"/>
+      <c r="G33" s="12"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B34" s="8" t="n">
         <v>25</v>
       </c>
-      <c r="C34" s="8" t="s">
+      <c r="C34" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="D34" s="12" t="s">
+      <c r="D34" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="E34" s="7" t="n">
+      <c r="E34" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="F34" s="7" t="s">
+      <c r="F34" s="8" t="s">
         <v>127</v>
       </c>
-      <c r="G34" s="8" t="s">
+      <c r="G34" s="9" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B35" s="7" t="n">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B35" s="8" t="n">
         <v>26</v>
       </c>
-      <c r="C35" s="8" t="s">
+      <c r="C35" s="9" t="s">
         <v>129</v>
       </c>
-      <c r="D35" s="12" t="s">
+      <c r="D35" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="E35" s="7" t="n">
+      <c r="E35" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="F35" s="7" t="s">
+      <c r="F35" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="G35" s="8" t="s">
+      <c r="G35" s="9" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B36" s="7" t="n">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B36" s="8" t="n">
         <v>27</v>
       </c>
-      <c r="C36" s="8" t="s">
+      <c r="C36" s="9" t="s">
         <v>132</v>
       </c>
-      <c r="D36" s="12" t="s">
+      <c r="D36" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="E36" s="7" t="n">
+      <c r="E36" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="F36" s="7" t="s">
+      <c r="F36" s="8" t="s">
         <v>133</v>
       </c>
-      <c r="G36" s="8" t="s">
+      <c r="G36" s="9" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B37" s="7" t="n">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B37" s="8" t="n">
         <v>28</v>
       </c>
-      <c r="C37" s="8" t="s">
+      <c r="C37" s="9" t="s">
         <v>135</v>
       </c>
-      <c r="D37" s="9" t="s">
+      <c r="D37" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="E37" s="7" t="n">
+      <c r="E37" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="F37" s="7" t="s">
+      <c r="F37" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="G37" s="8" t="s">
+      <c r="G37" s="9" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B38" s="7" t="n">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B38" s="8" t="n">
         <v>29</v>
       </c>
-      <c r="C38" s="8" t="s">
+      <c r="C38" s="9" t="s">
         <v>138</v>
       </c>
-      <c r="D38" s="9" t="s">
+      <c r="D38" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="E38" s="7" t="n">
+      <c r="E38" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="F38" s="7" t="s">
+      <c r="F38" s="8" t="s">
         <v>139</v>
       </c>
-      <c r="G38" s="8" t="s">
+      <c r="G38" s="9" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B39" s="7" t="n">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B39" s="8" t="n">
         <v>30</v>
       </c>
-      <c r="C39" s="8" t="s">
+      <c r="C39" s="9" t="s">
         <v>141</v>
       </c>
-      <c r="D39" s="13" t="s">
+      <c r="D39" s="17" t="s">
         <v>108</v>
       </c>
-      <c r="E39" s="7" t="n">
+      <c r="E39" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="F39" s="7" t="s">
+      <c r="F39" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="G39" s="8" t="s">
+      <c r="G39" s="9" t="s">
         <v>143</v>
       </c>
     </row>
@@ -2030,183 +2054,183 @@
   <dimension ref="B2:F15"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="3" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="3" style="1" width="14"/>
   </cols>
   <sheetData>
-    <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="1" t="s">
+    <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="4" t="s">
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B4" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="5" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="8" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B5" s="9" t="s">
         <v>150</v>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="C5" s="8" t="n">
         <v>7</v>
       </c>
-      <c r="D5" s="7" t="n">
+      <c r="D5" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="E5" s="7" t="n">
+      <c r="E5" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="10" t="n">
+      <c r="F5" s="11" t="n">
         <f aca="false">SUM(C5:E5)</f>
         <v>7</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="8" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B6" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C6" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="E6" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="F6" s="11" t="n">
+        <f aca="false">SUM(C6:E6)</f>
+        <v>65</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B7" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="C7" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="D6" s="7" t="n">
-        <v>21</v>
-      </c>
-      <c r="E6" s="7" t="n">
-        <v>50</v>
-      </c>
-      <c r="F6" s="10" t="n">
-        <f aca="false">SUM(C6:E6)</f>
-        <v>76</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="8" t="s">
-        <v>152</v>
-      </c>
-      <c r="C7" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="D7" s="7" t="n">
+      <c r="D7" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="7" t="n">
+      <c r="E7" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="F7" s="10" t="n">
+      <c r="F7" s="11" t="n">
         <f aca="false">SUM(C7:E7)</f>
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="8" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B8" s="9" t="s">
         <v>153</v>
       </c>
-      <c r="C8" s="7" t="n">
+      <c r="C8" s="8" t="n">
         <v>9</v>
       </c>
-      <c r="D8" s="7" t="n">
+      <c r="D8" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="E8" s="7" t="n">
+      <c r="E8" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="F8" s="10" t="n">
+      <c r="F8" s="11" t="n">
         <f aca="false">SUM(C8:E8)</f>
         <v>18</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="8" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B9" s="9" t="s">
         <v>154</v>
       </c>
-      <c r="C9" s="7" t="n">
+      <c r="C9" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="D9" s="7" t="n">
+      <c r="D9" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="E9" s="7" t="n">
+      <c r="E9" s="8" t="n">
         <v>10</v>
       </c>
-      <c r="F9" s="10" t="n">
+      <c r="F9" s="11" t="n">
         <f aca="false">SUM(C9:E9)</f>
         <v>10</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="14" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B10" s="18" t="s">
         <v>155</v>
       </c>
-      <c r="C10" s="15" t="n">
+      <c r="C10" s="19" t="n">
         <f aca="false">SUM(C5:C9)</f>
-        <v>29</v>
-      </c>
-      <c r="D10" s="15" t="n">
+        <v>24</v>
+      </c>
+      <c r="D10" s="19" t="n">
         <f aca="false">SUM(D5:D9)</f>
-        <v>26</v>
-      </c>
-      <c r="E10" s="15" t="n">
+        <v>17</v>
+      </c>
+      <c r="E10" s="19" t="n">
         <f aca="false">SUM(E5:E9)</f>
         <v>64</v>
       </c>
-      <c r="F10" s="15" t="n">
-        <f aca="false">SUM(F5:F9)</f>
-        <v>119</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="3" t="s">
+      <c r="F10" s="19" t="n">
+        <f aca="false">SUM(C10:E10)</f>
+        <v>105</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B12" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="16" t="s">
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
+      <c r="F12" s="4"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B13" s="20" t="s">
         <v>157</v>
       </c>
-      <c r="C13" s="16"/>
-      <c r="D13" s="16"/>
-      <c r="E13" s="16"/>
-      <c r="F13" s="16"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="17" t="s">
+      <c r="C13" s="20"/>
+      <c r="D13" s="20"/>
+      <c r="E13" s="20"/>
+      <c r="F13" s="20"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B14" s="21" t="s">
         <v>158</v>
       </c>
-      <c r="C14" s="17"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="17"/>
-      <c r="F14" s="17"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="2" t="s">
+      <c r="C14" s="21"/>
+      <c r="D14" s="21"/>
+      <c r="E14" s="21"/>
+      <c r="F14" s="21"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B15" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
+      <c r="C15" s="3"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>

<commit_message>
feat: remove client-side API keys — all AI calls route through Edge Function
Security hardening (Gap #4):
- Remove vestigial _apiKey params from ai.ts, embeddings.ts, rag.ts
- Remove anthropicKey/openAiKey from useChat options interface
- Remove EXPO_PUBLIC_ANTHROPIC_API_KEY and EXPO_PUBLIC_OPENAI_API_KEY
  constants from NavigatorScreen
- All AI calls (chat, classify, embed) now auth via Supabase JWT only
- Edge Function (ai-proxy) holds API keys server-side with prompt caching
- Zero TypeScript errors after refactor

Gap Analysis updated: #4 complete, P0 software gaps → 0 remaining hours

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Operations/Waypoint-GTM-Gap-Analysis-Mar2026.xlsx
+++ b/Operations/Waypoint-GTM-Gap-Analysis-Mar2026.xlsx
@@ -243,7 +243,7 @@
     <t xml:space="preserve">S2</t>
   </si>
   <si>
-    <t xml:space="preserve">Update ai.ts + embeddings.ts to call Supabase function URL</t>
+    <t xml:space="preserve">DONE — Client AI calls refactored to Edge Function proxy, API keys removed from client (Mar 15)</t>
   </si>
   <si>
     <t xml:space="preserve">Wire expo-document-picker for Document Vault uploads</t>
@@ -495,7 +495,7 @@
     <t xml:space="preserve">KEY INSIGHT</t>
   </si>
   <si>
-    <t xml:space="preserve">P0 items total ~19 hours. At 20 hrs/week, that's ~1 week to App Store submission readiness.</t>
+    <t xml:space="preserve">P0 items total ~15 hours. At 20 hrs/week, that's &lt;1 week to App Store submission readiness.</t>
   </si>
   <si>
     <t xml:space="preserve">P0 + P1 total ~31 hours. At 20 hrs/week, that's ~1.5 weeks — well within the June 8 deadline.</t>
@@ -1457,22 +1457,22 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="8" t="n">
+      <c r="B10" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="C10" s="15" t="s">
         <v>71</v>
       </c>
-      <c r="D10" s="13" t="s">
+      <c r="D10" s="14" t="s">
         <v>64</v>
       </c>
-      <c r="E10" s="8" t="n">
+      <c r="E10" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="F10" s="8" t="s">
+      <c r="F10" s="14" t="s">
         <v>72</v>
       </c>
-      <c r="G10" s="9" t="s">
+      <c r="G10" s="16" t="s">
         <v>73</v>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
         <v>151</v>
       </c>
       <c r="C6" s="8" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D6" s="8" t="n">
         <v>12</v>
@@ -2118,7 +2118,7 @@
       </c>
       <c r="F6" s="11" t="n">
         <f aca="false">SUM(C6:E6)</f>
-        <v>65</v>
+        <v>62</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2181,7 +2181,7 @@
       </c>
       <c r="C10" s="19" t="n">
         <f aca="false">SUM(C5:C9)</f>
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D10" s="19" t="n">
         <f aca="false">SUM(D5:D9)</f>
@@ -2193,7 +2193,7 @@
       </c>
       <c r="F10" s="19" t="n">
         <f aca="false">SUM(C10:E10)</f>
-        <v>105</v>
+        <v>102</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>